<commit_message>
updated moba analyses, removed multiple imputation and observed skills
</commit_message>
<xml_diff>
--- a/results/by_outcome/full_results_education_PGI.xlsx
+++ b/results/by_outcome/full_results_education_PGI.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Outcome</t>
   </si>
@@ -84,7 +84,13 @@
     <t xml:space="preserve">Upper</t>
   </si>
   <si>
+    <t xml:space="preserve">pval</t>
+  </si>
+  <si>
     <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diff</t>
   </si>
 </sst>
 </file>
@@ -468,32 +474,32 @@
         <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>0.636578570154257</v>
+        <v>0.654142655779591</v>
       </c>
       <c r="D2" t="n">
-        <v>0.363621994957094</v>
+        <v>0.345937238574254</v>
       </c>
       <c r="E2" t="n">
-        <v>1.00020056511135</v>
+        <v>1.00007989435384</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>
       <c r="H2"/>
       <c r="I2"/>
       <c r="J2" t="n">
-        <v>0.363549079695444</v>
+        <v>0.345909602350085</v>
       </c>
       <c r="K2" t="n">
-        <v>0.319632137220982</v>
+        <v>0.290386313364187</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0174156219765204</v>
+        <v>0.0178286943783974</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0462239887717918</v>
+        <v>0.05062144762764</v>
       </c>
       <c r="N2" t="n">
-        <v>0.337047759197502</v>
+        <v>0.308215007742584</v>
       </c>
       <c r="O2"/>
     </row>
@@ -508,10 +514,10 @@
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="n">
-        <v>0.607764425405691</v>
+        <v>0.621347282574517</v>
       </c>
       <c r="G3" t="n">
-        <v>0.319696244276175</v>
+        <v>0.290409513591059</v>
       </c>
       <c r="H3"/>
       <c r="I3"/>
@@ -535,10 +541,10 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4" t="n">
-        <v>0.59034531046301</v>
+        <v>0.603517163784102</v>
       </c>
       <c r="I4" t="n">
-        <v>0.295417105285085</v>
+        <v>0.246962367415101</v>
       </c>
       <c r="J4"/>
       <c r="K4"/>
@@ -546,7 +552,7 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4" t="n">
-        <v>0.409773068467235</v>
+        <v>0.396531049977725</v>
       </c>
     </row>
   </sheetData>
@@ -579,6 +585,9 @@
       <c r="F1" t="s">
         <v>23</v>
       </c>
+      <c r="G1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -588,16 +597,19 @@
         <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>0.363549079695444</v>
+        <v>0.345909602350085</v>
       </c>
       <c r="D2" t="n">
-        <v>0.323649873116815</v>
+        <v>0.314293271650187</v>
       </c>
       <c r="E2" t="n">
-        <v>0.403448286274072</v>
+        <v>0.375568872004405</v>
       </c>
       <c r="F2" t="n">
-        <v>1814</v>
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4334</v>
       </c>
     </row>
     <row r="3">
@@ -608,16 +620,19 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>0.337047759197502</v>
+        <v>0.308215007742584</v>
       </c>
       <c r="D3" t="n">
-        <v>0.294393425645801</v>
+        <v>0.27779039847751</v>
       </c>
       <c r="E3" t="n">
-        <v>0.379702092749204</v>
+        <v>0.340443124402345</v>
       </c>
       <c r="F3" t="n">
-        <v>1814</v>
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4334</v>
       </c>
     </row>
     <row r="4">
@@ -628,16 +643,42 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>0.409773068467235</v>
+        <v>0.396531049977725</v>
       </c>
       <c r="D4" t="n">
-        <v>0.371958556475419</v>
+        <v>0.364255360270343</v>
       </c>
       <c r="E4" t="n">
-        <v>0.447587580459052</v>
+        <v>0.429280996298816</v>
       </c>
       <c r="F4" t="n">
-        <v>1814</v>
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.088316042235141</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0751171238363021</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.103003265167507</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rename scripts to reflect pipeline order; remove unused result files
- Renamed R scripts with numbered prefixes matching execution order
  (GENDER_MAIN, GENDER_IMPUT, COMBINE_MOBA, FIGURES → 03–08)
- Deleted superseded scripts (01_CLEAN_DATA_single_outcomes, PGIs,
  04_DESCRIPTIVES, 05_GRAPHS_PRESENTATIONS)
- Removed stale results: old naming conventions (sons/daughters, no
  sample suffix), inactive outcomes (income, wealth, health), and
  observed natural talent variants

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/by_outcome/full_results_education_PGI.xlsx
+++ b/results/by_outcome/full_results_education_PGI.xlsx
@@ -474,32 +474,32 @@
         <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>0.654142655779591</v>
+        <v>0.662718487922359</v>
       </c>
       <c r="D2" t="n">
-        <v>0.345937238574254</v>
+        <v>0.337359370384728</v>
       </c>
       <c r="E2" t="n">
-        <v>1.00007989435384</v>
+        <v>1.00007785830709</v>
       </c>
       <c r="F2"/>
       <c r="G2"/>
       <c r="H2"/>
       <c r="I2"/>
       <c r="J2" t="n">
-        <v>0.345909602350085</v>
+        <v>0.337333106200155</v>
       </c>
       <c r="K2" t="n">
-        <v>0.290386313364187</v>
+        <v>0.283376534543844</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0178286943783974</v>
+        <v>0.0155418175011335</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05062144762764</v>
+        <v>0.0486991907913854</v>
       </c>
       <c r="N2" t="n">
-        <v>0.308215007742584</v>
+        <v>0.298918352044978</v>
       </c>
       <c r="O2"/>
     </row>
@@ -514,10 +514,10 @@
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="n">
-        <v>0.621347282574517</v>
+        <v>0.629558533055156</v>
       </c>
       <c r="G3" t="n">
-        <v>0.290409513591059</v>
+        <v>0.283398597761092</v>
       </c>
       <c r="H3"/>
       <c r="I3"/>
@@ -541,10 +541,10 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4" t="n">
-        <v>0.603517163784102</v>
+        <v>0.614015505494422</v>
       </c>
       <c r="I4" t="n">
-        <v>0.246962367415101</v>
+        <v>0.241862644105105</v>
       </c>
       <c r="J4"/>
       <c r="K4"/>
@@ -552,7 +552,7 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4" t="n">
-        <v>0.396531049977725</v>
+        <v>0.38603229699154</v>
       </c>
     </row>
   </sheetData>
@@ -597,13 +597,13 @@
         <v>15</v>
       </c>
       <c r="C2" t="n">
-        <v>0.345909602350085</v>
+        <v>0.337333106200155</v>
       </c>
       <c r="D2" t="n">
-        <v>0.314293271650187</v>
+        <v>0.309733067430175</v>
       </c>
       <c r="E2" t="n">
-        <v>0.375568872004405</v>
+        <v>0.362817553901207</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -620,13 +620,13 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>0.308215007742584</v>
+        <v>0.298918352044978</v>
       </c>
       <c r="D3" t="n">
-        <v>0.27779039847751</v>
+        <v>0.274662989455965</v>
       </c>
       <c r="E3" t="n">
-        <v>0.340443124402345</v>
+        <v>0.332622860092453</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -643,13 +643,13 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>0.396531049977725</v>
+        <v>0.38603229699154</v>
       </c>
       <c r="D4" t="n">
-        <v>0.364255360270343</v>
+        <v>0.364451789385342</v>
       </c>
       <c r="E4" t="n">
-        <v>0.429280996298816</v>
+        <v>0.420605427034511</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -666,13 +666,13 @@
         <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.088316042235141</v>
+        <v>0.0871139449465624</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0751171238363021</v>
+        <v>0.0741205556809228</v>
       </c>
       <c r="E5" t="n">
-        <v>0.103003265167507</v>
+        <v>0.100099786593869</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add bootstrap SE to output and fix CI/SE consistency
- Add SE column (sd of bootstrap samples) directly to compute_indexes_bootstrap output
- Remove redundant first line in est_fun cluster resampling
- Fix setwd paths in 00_MASTER.R and 06_DESCRIPTIVES.R
- Update 06_DESCRIPTIVES.R to use SE directly instead of back-calculating from CIs
- Add SE approximation for MoBa hardcoded data in 07_COMBINE_MOBA.R
- Revert p-value to normal approximation (z = estimate/se_boot) for precision
- Regenerate all results files with updated pipeline

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/by_outcome/full_results_education_PGI.xlsx
+++ b/results/by_outcome/full_results_education_PGI.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">Outcome</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t xml:space="preserve">Estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE</t>
   </si>
   <si>
     <t xml:space="preserve">Lower</t>
@@ -588,6 +591,9 @@
       <c r="G1" t="s">
         <v>24</v>
       </c>
+      <c r="H1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -600,15 +606,18 @@
         <v>0.337333106200155</v>
       </c>
       <c r="D2" t="n">
+        <v>0.0132130211612754</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.309733067430175</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.362817553901207</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>4334</v>
       </c>
     </row>
@@ -623,15 +632,18 @@
         <v>0.298918352044978</v>
       </c>
       <c r="D3" t="n">
+        <v>0.0153491485707949</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.274662989455965</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.332622860092453</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>4334</v>
       </c>
     </row>
@@ -646,21 +658,24 @@
         <v>0.38603229699154</v>
       </c>
       <c r="D4" t="n">
+        <v>0.0147049798413089</v>
+      </c>
+      <c r="E4" t="n">
         <v>0.364451789385342</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.420605427034511</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>4334</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -669,15 +684,18 @@
         <v>0.0871139449465624</v>
       </c>
       <c r="D5" t="n">
+        <v>0.00737191150207233</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.0741205556809228</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.100099786593869</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>4334</v>
       </c>
     </row>

</xml_diff>

<commit_message>
appendix figure with one PGI at the time
</commit_message>
<xml_diff>
--- a/results/by_outcome/full_results_education_PGI.xlsx
+++ b/results/by_outcome/full_results_education_PGI.xlsx
@@ -493,16 +493,16 @@
         <v>0.337333106200155</v>
       </c>
       <c r="K2" t="n">
-        <v>0.283376534543844</v>
+        <v>0.284595000820937</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0155418175011335</v>
+        <v>0.0175496575937104</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0486991907913854</v>
+        <v>0.051438890469951</v>
       </c>
       <c r="N2" t="n">
-        <v>0.298918352044978</v>
+        <v>0.302144658414648</v>
       </c>
       <c r="O2"/>
     </row>
@@ -517,10 +517,10 @@
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="n">
-        <v>0.629558533055156</v>
+        <v>0.628826616487818</v>
       </c>
       <c r="G3" t="n">
-        <v>0.283398597761092</v>
+        <v>0.284617158905907</v>
       </c>
       <c r="H3"/>
       <c r="I3"/>
@@ -544,10 +544,10 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4" t="n">
-        <v>0.614015505494422</v>
+        <v>0.611275592507478</v>
       </c>
       <c r="I4" t="n">
-        <v>0.241862644105105</v>
+        <v>0.242319883930301</v>
       </c>
       <c r="J4"/>
       <c r="K4"/>
@@ -555,7 +555,7 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4" t="n">
-        <v>0.38603229699154</v>
+        <v>0.388771996670106</v>
       </c>
     </row>
   </sheetData>
@@ -629,16 +629,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>0.298918352044978</v>
+        <v>0.302144658414648</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0160234137057634</v>
+        <v>0.015514238714371</v>
       </c>
       <c r="E3" t="n">
-        <v>0.268084514133279</v>
+        <v>0.270928657299641</v>
       </c>
       <c r="F3" t="n">
-        <v>0.33039133258701</v>
+        <v>0.331955663264731</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -655,16 +655,16 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>0.38603229699154</v>
+        <v>0.388771996670106</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0161203054352775</v>
+        <v>0.0158013127038112</v>
       </c>
       <c r="E4" t="n">
-        <v>0.353492396445637</v>
+        <v>0.356708206676253</v>
       </c>
       <c r="F4" t="n">
-        <v>0.419616469277901</v>
+        <v>0.420723564457306</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -681,16 +681,16 @@
         <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0871139449465624</v>
+        <v>0.0866273382554584</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0072613277840819</v>
+        <v>0.00702358497127891</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0742087011588903</v>
+        <v>0.0739236353837278</v>
       </c>
       <c r="F5" t="n">
-        <v>0.101534513229491</v>
+        <v>0.100636638039421</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Herd et al replication, removed PGI wellbeing, 500 iterations, final power analysys and PGI correction figures
</commit_message>
<xml_diff>
--- a/results/by_outcome/full_results_education_PGI.xlsx
+++ b/results/by_outcome/full_results_education_PGI.xlsx
@@ -493,16 +493,16 @@
         <v>0.337333106200155</v>
       </c>
       <c r="K2" t="n">
-        <v>0.284595000820937</v>
+        <v>0.285085911510983</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0175496575937104</v>
+        <v>0.0165237392114518</v>
       </c>
       <c r="M2" t="n">
-        <v>0.051438890469951</v>
+        <v>0.0474865193043971</v>
       </c>
       <c r="N2" t="n">
-        <v>0.302144658414648</v>
+        <v>0.301609650722435</v>
       </c>
       <c r="O2"/>
     </row>
@@ -517,10 +517,10 @@
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="n">
-        <v>0.628826616487818</v>
+        <v>0.631753297119773</v>
       </c>
       <c r="G3" t="n">
-        <v>0.284617158905907</v>
+        <v>0.285108107817428</v>
       </c>
       <c r="H3"/>
       <c r="I3"/>
@@ -544,10 +544,10 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4" t="n">
-        <v>0.611275592507478</v>
+        <v>0.61522827139796</v>
       </c>
       <c r="I4" t="n">
-        <v>0.242319883930301</v>
+        <v>0.245953227331713</v>
       </c>
       <c r="J4"/>
       <c r="K4"/>
@@ -555,7 +555,7 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4" t="n">
-        <v>0.388771996670106</v>
+        <v>0.384819625504552</v>
       </c>
     </row>
   </sheetData>
@@ -606,13 +606,13 @@
         <v>0.337333106200155</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0150222214200847</v>
+        <v>0.0156913804298284</v>
       </c>
       <c r="E2" t="n">
-        <v>0.307938690709166</v>
+        <v>0.309381231278446</v>
       </c>
       <c r="F2" t="n">
-        <v>0.367585993307718</v>
+        <v>0.369659457272415</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -629,16 +629,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>0.302144658414648</v>
+        <v>0.301609650722435</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0154827622246759</v>
+        <v>0.0142728177383851</v>
       </c>
       <c r="E3" t="n">
-        <v>0.271958592247215</v>
+        <v>0.27529088284028</v>
       </c>
       <c r="F3" t="n">
-        <v>0.333205626874508</v>
+        <v>0.32960806761775</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -655,16 +655,16 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>0.388771996670106</v>
+        <v>0.384819625504552</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0156921403726395</v>
+        <v>0.014747473090196</v>
       </c>
       <c r="E4" t="n">
-        <v>0.360151037552612</v>
+        <v>0.357145105772558</v>
       </c>
       <c r="F4" t="n">
-        <v>0.420965924106323</v>
+        <v>0.413518188546051</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -681,16 +681,16 @@
         <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0866273382554584</v>
+        <v>0.0832099747821175</v>
       </c>
       <c r="D5" t="n">
-        <v>0.00697855261667966</v>
+        <v>0.00661655288163531</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0739034288670258</v>
+        <v>0.0722643159261203</v>
       </c>
       <c r="F5" t="n">
-        <v>0.100540687034918</v>
+        <v>0.0973304319238288</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>

</xml_diff>